<commit_message>
Simplify data cleaning and pipeline helpers
Remove obsolete Spanish plan column compatibility.
Remove rehearsal time translation.
Inline best plan summary printing.
</commit_message>
<xml_diff>
--- a/outputs/worship_planning_2026-01-04_2026-06-28.xlsx
+++ b/outputs/worship_planning_2026-01-04_2026-06-28.xlsx
@@ -486,33 +486,37 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Gabriel Romero</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sofía Medina</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Tomás Ortega</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Samuel Molina</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Samuel Ortega</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Daniel Herrera</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Thomas Walker</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Lucia Mendoza</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Matthew Turner</t>
+          <t>Lucía Rojas</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
     </row>
@@ -530,28 +534,32 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Isabella Palacios</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bruno Vega</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Mateo Cabrera</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>Valentina Salazar</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Camila Miranda</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Bruno Vega</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Matthew Brooks</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Valentina Fuentes</t>
+          <t>Mateo Santos</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -574,35 +582,31 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Samuel Ortega</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Daniel Herrera</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mariana Campos</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Samuel Molina</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Mariana Campos</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Gabriel Romero</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Lucy Bennett</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Samuel Molina</t>
-        </is>
-      </c>
+          <t>Daniel Herrera</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -618,7 +622,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -633,13 +637,13 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Matthew Brooks</t>
+          <t>Mateo Cabrera</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Nicholas Reed</t>
+          <t>Nicolás Mendoza</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -662,7 +666,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Thomas Walker</t>
+          <t>Samuel Molina</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -672,22 +676,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Mariana Campos</t>
+          <t>Tomás Ortega</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lucia Mendoza</t>
+          <t>Lucía Mendoza</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Samuel Ortega</t>
+          <t>Gabriel Romero</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Matthew Turner</t>
+          <t>Valentina Fuentes</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -710,32 +714,32 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>Bruno Vega</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Nicolás Mendoza</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Mateo Cabrera</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Valentina Salazar</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>Isabella Palacios</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Camila Miranda</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Bruno Vega</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Matthew Brooks</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Valentina Salazar</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Nicholas Reed</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -758,17 +762,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Gabriel Romero</t>
+          <t>Tomás Ortega</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Thomas Walker</t>
+          <t>Mariana Campos</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -783,12 +787,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Lucy Bennett</t>
+          <t>Lucía Rojas</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
     </row>
@@ -806,33 +810,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>Mateo Cabrera</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>Bruno Vega</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Daniel Herrera</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Nicholas Reed</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Matthew Brooks</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Matthew Turner</t>
+          <t>Mateo Santos</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
     </row>
@@ -850,14 +850,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>Daniel Herrera</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>Valentina Fuentes</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Camila Miranda</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>Mariana Campos</t>
@@ -865,13 +865,13 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Lucia Mendoza</t>
+          <t>Lucía Mendoza</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Valentina Fuentes</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -890,25 +890,25 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Matthew Brooks</t>
+          <t>Valentina Salazar</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Thomas Walker</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Valentina Salazar</t>
-        </is>
-      </c>
+          <t>Tomás Ortega</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Mateo Cabrera</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>Isabella Palacios</t>
@@ -916,7 +916,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
     </row>
@@ -934,12 +934,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Lucy Bennett</t>
+          <t>Lucía Rojas</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -952,19 +952,15 @@
           <t>Samuel Molina</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Gabriel Romero</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Matthew Turner</t>
+          <t>Mateo Santos</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
     </row>
@@ -982,12 +978,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nicholas Reed</t>
+          <t>Nicolás Mendoza</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -997,7 +993,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Matthew Brooks</t>
+          <t>Mateo Cabrera</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1008,7 +1004,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
     </row>
@@ -1026,12 +1022,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Samuel Molina</t>
+          <t>Valentina Fuentes</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1041,20 +1037,16 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lucia Mendoza</t>
+          <t>Lucía Mendoza</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Valentina Fuentes</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Sophia Carter</t>
-        </is>
-      </c>
+          <t>Sofía Medina</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1070,33 +1062,37 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>Gabriel Romero</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Tomás Ortega</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Samuel Molina</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>Samuel Ortega</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Daniel Herrera</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Thomas Walker</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Matthew Brooks</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Matthew Turner</t>
+          <t>Mateo Santos</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
     </row>
@@ -1114,29 +1110,37 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>Isabella Palacios</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Daniel Herrera</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Bruno Vega</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Mateo Cabrera</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Valentina Salazar</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Camila Miranda</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Bruno Vega</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Isabella Palacios</t>
+          <t>Nicolás Mendoza</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
     </row>
@@ -1154,37 +1158,33 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Samuel Ortega</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Mariana Campos</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>Samuel Molina</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Mariana Campos</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Matthew Brooks</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Gabriel Romero</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Lucy Bennett</t>
+          <t>Lucía Rojas</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Samuel Molina</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
     </row>
@@ -1202,12 +1202,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1215,16 +1215,20 @@
           <t>Bruno Vega</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Mateo Cabrera</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Nicholas Reed</t>
+          <t>Valentina Fuentes</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
     </row>
@@ -1242,22 +1246,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Thomas Walker</t>
+          <t>Samuel Molina</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Mariana Campos</t>
+          <t>Tomás Ortega</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Lucia Mendoza</t>
+          <t>Lucía Mendoza</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1267,12 +1271,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Matthew Turner</t>
+          <t>Mateo Santos</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
     </row>
@@ -1290,37 +1294,37 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
+          <t>Bruno Vega</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Daniel Herrera</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Nicolás Mendoza</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Mateo Cabrera</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Valentina Salazar</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>Isabella Palacios</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Camila Miranda</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Bruno Vega</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Matthew Brooks</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Valentina Salazar</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Nicholas Reed</t>
-        </is>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
     </row>
@@ -1338,37 +1342,37 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>Tomás Ortega</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Mariana Campos</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Samuel Molina</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>Gabriel Romero</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Daniel Herrera</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Thomas Walker</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Samuel Molina</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Samuel Ortega</t>
-        </is>
-      </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Lucy Bennett</t>
+          <t>Lucía Rojas</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
     </row>
@@ -1386,33 +1390,29 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
+          <t>Mateo Cabrera</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sofía Medina</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>Bruno Vega</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Sophia Carter</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Nicholas Reed</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Matthew Brooks</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Matthew Turner</t>
+          <t>Valentina Fuentes</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Valentina Fuentes</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1440,12 +1440,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Mariana Campos</t>
+          <t>Tomás Ortega</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Lucia Mendoza</t>
+          <t>Lucía Mendoza</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1455,10 +1455,14 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
+          <t>Mateo Santos</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -1474,25 +1478,21 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Matthew Brooks</t>
+          <t>Valentina Salazar</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Mateo Cabrera</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Thomas Walker</t>
+          <t>Bruno Vega</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Valentina Salazar</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>Isabella Palacios</t>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Mateo Cabrera</t>
         </is>
       </c>
     </row>
@@ -1518,12 +1518,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Lucy Bennett</t>
+          <t>Lucía Rojas</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sophia Carter</t>
+          <t>Sofía Medina</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1538,19 +1538,15 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Gabriel Romero</t>
+          <t>Samuel Ortega</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Matthew Turner</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Sophia Carter</t>
-        </is>
-      </c>
+          <t>Sofía Medina</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -1566,7 +1562,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Nicholas Reed</t>
+          <t>Nicolás Mendoza</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1576,18 +1572,18 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Bruno Vega</t>
+          <t>Tomás Ortega</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Matthew Brooks</t>
+          <t>Mateo Cabrera</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Isabella Palacios</t>
+          <t>Mateo Santos</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1610,7 +1606,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Samuel Molina</t>
+          <t>Valentina Fuentes</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1625,20 +1621,16 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Lucia Mendoza</t>
+          <t>Lucía Mendoza</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Valentina Fuentes</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
           <t>Daniel Herrera</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add monthly plan view and dashboard previews
- Add a monthly HTML plan view grouped by service month and embed it in the Streamlit dashboard.
- Update the README with dashboard screenshots and refreshed feature descriptions.
- Rename generated planning option files to sequential plan IDs and refresh demo artifacts.
- Centralize planning schema constants and remove legacy plan column aliases.
- Improve dashboard comparison UX with ranking labels, winner highlighting, ordered charts, and integer availability axes.
- Remove unused Pillow dependency.
</commit_message>
<xml_diff>
--- a/outputs/worship_planning_2026-01-04_2026-06-28.xlsx
+++ b/outputs/worship_planning_2026-01-04_2026-06-28.xlsx
@@ -491,12 +491,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Thomas Walker</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -511,12 +511,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Lucía Rojas</t>
+          <t>Lucy Bennett</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -559,12 +559,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Mateo Santos</t>
+          <t>Matthew Turner</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -603,7 +603,7 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -622,12 +622,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -637,18 +637,18 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Nicolás Mendoza</t>
+          <t>Nicholas Reed</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
     </row>
@@ -666,27 +666,27 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Samuel Molina</t>
+          <t>Thomas Walker</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Mariana Campos</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lucía Mendoza</t>
+          <t>Lucia Mendoza</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Gabriel Romero</t>
+          <t>Samuel Ortega</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
     </row>
@@ -719,17 +719,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Nicolás Mendoza</t>
+          <t>Nicholas Reed</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -739,12 +739,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Isabella Palacios</t>
+          <t>Matthew Turner</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Lucy Bennett</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -782,19 +782,15 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Samuel Ortega</t>
+          <t>Gabriel Romero</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Lucía Rojas</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Sofía Medina</t>
-        </is>
-      </c>
+          <t>Sophia Carter</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -810,7 +806,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -820,14 +816,14 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bruno Vega</t>
+          <t>Thomas Walker</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Mateo Santos</t>
+          <t>Isabella Palacios</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -865,16 +861,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Lucía Mendoza</t>
+          <t>Lucia Mendoza</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
+          <t>Matthew Turner</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>Valentina Fuentes</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -895,28 +895,28 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Bruno Vega</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Isabella Palacios</t>
+          <t>Nicholas Reed</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Lucía Rojas</t>
+          <t>Samuel Molina</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -944,18 +944,18 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Mariana Campos</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Samuel Molina</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>Thomas Walker</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Samuel Ortega</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Mateo Santos</t>
+          <t>Lucy Bennett</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nicolás Mendoza</t>
+          <t>Nicholas Reed</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1037,16 +1037,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lucía Mendoza</t>
+          <t>Lucia Mendoza</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
+          <t>Matthew Turner</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Sophia Carter</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1072,7 +1076,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Thomas Walker</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1087,7 +1091,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Mateo Santos</t>
+          <t>Lucy Bennett</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1125,7 +1129,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1135,7 +1139,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Nicolás Mendoza</t>
+          <t>Nicholas Reed</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1179,7 +1183,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Lucía Rojas</t>
+          <t>Matthew Turner</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1202,7 +1206,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1217,7 +1221,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -1246,7 +1250,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Samuel Molina</t>
+          <t>Thomas Walker</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1256,12 +1260,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Mariana Campos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Lucía Mendoza</t>
+          <t>Lucia Mendoza</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1271,14 +1275,10 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Mateo Santos</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Camila Miranda</t>
-        </is>
-      </c>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Nicolás Mendoza</t>
+          <t>Nicholas Reed</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Lucy Bennett</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Lucía Rojas</t>
+          <t>Matthew Turner</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
     </row>
@@ -1440,12 +1440,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Thomas Walker</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Lucía Mendoza</t>
+          <t>Lucia Mendoza</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1455,14 +1455,10 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Mateo Santos</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Camila Miranda</t>
-        </is>
-      </c>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -1483,7 +1479,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1500,7 +1496,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
     </row>
@@ -1518,12 +1514,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Lucía Rojas</t>
+          <t>Samuel Molina</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
+          <t>Sophia Carter</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1531,11 +1527,7 @@
           <t>Mariana Campos</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Samuel Molina</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Samuel Ortega</t>
@@ -1543,10 +1535,14 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Sofía Medina</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
+          <t>Matthew Turner</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Sophia Carter</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -1562,33 +1558,33 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Nicolás Mendoza</t>
+          <t>Nicholas Reed</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Tomás Ortega</t>
+          <t>Thomas Walker</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Mateo Cabrera</t>
+          <t>Matthew Brooks</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Mateo Santos</t>
+          <t>Isabella Palacios</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Camila Miranda</t>
+          <t>Daniel Herrera</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1607,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
+          <t>Camila Miranda</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1621,16 +1617,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Lucía Mendoza</t>
+          <t>Lucia Mendoza</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Daniel Herrera</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
+          <t>Lucy Bennett</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Camila Miranda</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>